<commit_message>
fixed dublicates when export_employee, changed template
</commit_message>
<xml_diff>
--- a/employee_list.xlsx
+++ b/employee_list.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t xml:space="preserve">社員番号</t>
   </si>
@@ -118,6 +118,72 @@
   </si>
   <si>
     <t>sarvarbekfozilov59@gmail.com</t>
+  </si>
+  <si>
+    <t>sda</t>
+  </si>
+  <si>
+    <t>wdadwada</t>
+  </si>
+  <si>
+    <t>ewqeqw</t>
+  </si>
+  <si>
+    <t>department2</t>
+  </si>
+  <si>
+    <t>position2</t>
+  </si>
+  <si>
+    <t>543534</t>
+  </si>
+  <si>
+    <t>gulnazmambetlepesova19@gmail.com</t>
+  </si>
+  <si>
+    <t>dsadsad</t>
+  </si>
+  <si>
+    <t>sadas</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>position</t>
+  </si>
+  <si>
+    <t>231321321</t>
+  </si>
+  <si>
+    <t>islom@gmail.com</t>
+  </si>
+  <si>
+    <t>DK0009</t>
+  </si>
+  <si>
+    <t>sadsad</t>
+  </si>
+  <si>
+    <t>123123</t>
+  </si>
+  <si>
+    <t>8999259914</t>
+  </si>
+  <si>
+    <t>210042r@jdu.uz</t>
+  </si>
+  <si>
+    <t>toxtar</t>
+  </si>
+  <si>
+    <t>justfordota08@gmail.com</t>
+  </si>
+  <si>
+    <t>department3</t>
+  </si>
+  <si>
+    <t>gulnazmambetlepesova@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -634,16 +700,16 @@
     </row>
     <row r="2" ht="12.8">
       <c r="A2" s="6" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>14</v>
@@ -652,30 +718,30 @@
         <v>15</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" ht="12.8">
       <c r="A3" s="6" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>14</v>
@@ -684,30 +750,30 @@
         <v>15</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" ht="12.8">
       <c r="A4" s="6" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>14</v>
@@ -716,21 +782,21 @@
         <v>15</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="12.8">
       <c r="A5" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>11</v>
@@ -739,7 +805,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>14</v>
@@ -748,28 +814,49 @@
         <v>15</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="I5" s="10" t="s">
         <v>30</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" ht="12.8">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="7"/>
+      <c r="A6" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="7" ht="12.8">
       <c r="A7" s="6"/>
@@ -1750,80 +1837,14 @@
       <c r="I95" s="10"/>
       <c r="J95" s="7"/>
     </row>
-    <row r="96" ht="12.8">
-      <c r="A96" s="6"/>
-      <c r="B96" s="7"/>
-      <c r="C96" s="7"/>
-      <c r="D96" s="7"/>
-      <c r="E96" s="7"/>
-      <c r="G96" s="8"/>
-      <c r="H96" s="9"/>
-      <c r="I96" s="10"/>
-      <c r="J96" s="7"/>
-    </row>
-    <row r="97" ht="12.8">
-      <c r="A97" s="6"/>
-      <c r="B97" s="7"/>
-      <c r="C97" s="7"/>
-      <c r="D97" s="7"/>
-      <c r="E97" s="7"/>
-      <c r="G97" s="8"/>
-      <c r="H97" s="9"/>
-      <c r="I97" s="10"/>
-      <c r="J97" s="7"/>
-    </row>
-    <row r="98" ht="12.8">
-      <c r="A98" s="6"/>
-      <c r="B98" s="7"/>
-      <c r="C98" s="7"/>
-      <c r="D98" s="7"/>
-      <c r="E98" s="7"/>
-      <c r="G98" s="8"/>
-      <c r="H98" s="9"/>
-      <c r="I98" s="10"/>
-      <c r="J98" s="7"/>
-    </row>
-    <row r="99" ht="12.8">
-      <c r="A99" s="6"/>
-      <c r="B99" s="7"/>
-      <c r="C99" s="7"/>
-      <c r="D99" s="7"/>
-      <c r="E99" s="7"/>
-      <c r="G99" s="8"/>
-      <c r="H99" s="9"/>
-      <c r="I99" s="10"/>
-      <c r="J99" s="7"/>
-    </row>
-    <row r="100" ht="12.8">
-      <c r="A100" s="6"/>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="7"/>
-      <c r="G100" s="8"/>
-      <c r="H100" s="9"/>
-      <c r="I100" s="10"/>
-      <c r="J100" s="7"/>
-    </row>
-    <row r="101" ht="12.8">
-      <c r="A101" s="6"/>
-      <c r="B101" s="7"/>
-      <c r="C101" s="7"/>
-      <c r="D101" s="7"/>
-      <c r="E101" s="7"/>
-      <c r="G101" s="8"/>
-      <c r="H101" s="9"/>
-      <c r="I101" s="10"/>
-      <c r="J101" s="7"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G101" type="list">
-      <formula1>部署!$A$2:$A1000</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G95" type="list">
+      <formula1>部署!$A$2:$A999</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H101" type="list">
-      <formula1>役職!$A$2:$A1000</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H95" type="list">
+      <formula1>役職!$A$2:$A999</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1852,14 +1873,18 @@
     </row>
     <row r="2" ht="13.8">
       <c r="A2" s="12" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" ht="13.8">
-      <c r="A3" s="12"/>
-    </row>
-    <row r="4" ht="13.8">
-      <c r="A4" s="12"/>
+      <c r="A3" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="true">
+      <c r="A4" s="13" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="true">
       <c r="A5" s="13"/>
@@ -1887,9 +1912,6 @@
     </row>
     <row r="13" ht="15.75" customHeight="true">
       <c r="A13" s="13"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="true">
-      <c r="A14" s="13"/>
     </row>
   </sheetData>
   <printOptions gridLinesSet="true"/>
@@ -1917,14 +1939,18 @@
     </row>
     <row r="2" ht="13.8">
       <c r="A2" s="14" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="12.8">
-      <c r="A3" s="1"/>
-    </row>
-    <row r="4" ht="12.8">
-      <c r="A4" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="true">
+      <c r="A4" s="1" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="5" ht="15.75" customHeight="true">
       <c r="A5" s="1"/>
@@ -1946,9 +1972,6 @@
     </row>
     <row r="11" ht="15.75" customHeight="true">
       <c r="A11" s="1"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="true">
-      <c r="A12" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLinesSet="true"/>

</xml_diff>

<commit_message>
fixed export employee showing admins
</commit_message>
<xml_diff>
--- a/employee_list.xlsx
+++ b/employee_list.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t xml:space="preserve">社員番号</t>
   </si>
@@ -184,6 +184,21 @@
   </si>
   <si>
     <t>gulnazmambetlepesova@gmail.com</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>Admin05</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>512334</t>
+  </si>
+  <si>
+    <t>admin@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -712,7 +727,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>15</v>
@@ -828,46 +843,67 @@
     </row>
     <row r="6" ht="12.8">
       <c r="A6" s="6" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" ht="12.8">
+      <c r="A7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I7" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J7" s="7" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" ht="12.8">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="7"/>
     </row>
     <row r="8" ht="12.8">
       <c r="A8" s="6"/>
@@ -1672,179 +1708,14 @@
       <c r="I80" s="10"/>
       <c r="J80" s="7"/>
     </row>
-    <row r="81" ht="12.8">
-      <c r="A81" s="6"/>
-      <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="7"/>
-      <c r="E81" s="7"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="9"/>
-      <c r="I81" s="10"/>
-      <c r="J81" s="7"/>
-    </row>
-    <row r="82" ht="12.8">
-      <c r="A82" s="6"/>
-      <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
-      <c r="D82" s="7"/>
-      <c r="E82" s="7"/>
-      <c r="G82" s="8"/>
-      <c r="H82" s="9"/>
-      <c r="I82" s="10"/>
-      <c r="J82" s="7"/>
-    </row>
-    <row r="83" ht="12.8">
-      <c r="A83" s="6"/>
-      <c r="B83" s="7"/>
-      <c r="C83" s="7"/>
-      <c r="D83" s="7"/>
-      <c r="E83" s="7"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="9"/>
-      <c r="I83" s="10"/>
-      <c r="J83" s="7"/>
-    </row>
-    <row r="84" ht="12.8">
-      <c r="A84" s="6"/>
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="9"/>
-      <c r="I84" s="10"/>
-      <c r="J84" s="7"/>
-    </row>
-    <row r="85" ht="12.8">
-      <c r="A85" s="6"/>
-      <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
-      <c r="D85" s="7"/>
-      <c r="E85" s="7"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="9"/>
-      <c r="I85" s="10"/>
-      <c r="J85" s="7"/>
-    </row>
-    <row r="86" ht="12.8">
-      <c r="A86" s="6"/>
-      <c r="B86" s="7"/>
-      <c r="C86" s="7"/>
-      <c r="D86" s="7"/>
-      <c r="E86" s="7"/>
-      <c r="G86" s="8"/>
-      <c r="H86" s="9"/>
-      <c r="I86" s="10"/>
-      <c r="J86" s="7"/>
-    </row>
-    <row r="87" ht="12.8">
-      <c r="A87" s="6"/>
-      <c r="B87" s="7"/>
-      <c r="C87" s="7"/>
-      <c r="D87" s="7"/>
-      <c r="E87" s="7"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="9"/>
-      <c r="I87" s="10"/>
-      <c r="J87" s="7"/>
-    </row>
-    <row r="88" ht="12.8">
-      <c r="A88" s="6"/>
-      <c r="B88" s="7"/>
-      <c r="C88" s="7"/>
-      <c r="D88" s="7"/>
-      <c r="E88" s="7"/>
-      <c r="G88" s="8"/>
-      <c r="H88" s="9"/>
-      <c r="I88" s="10"/>
-      <c r="J88" s="7"/>
-    </row>
-    <row r="89" ht="12.8">
-      <c r="A89" s="6"/>
-      <c r="B89" s="7"/>
-      <c r="C89" s="7"/>
-      <c r="D89" s="7"/>
-      <c r="E89" s="7"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="9"/>
-      <c r="I89" s="10"/>
-      <c r="J89" s="7"/>
-    </row>
-    <row r="90" ht="12.8">
-      <c r="A90" s="6"/>
-      <c r="B90" s="7"/>
-      <c r="C90" s="7"/>
-      <c r="D90" s="7"/>
-      <c r="E90" s="7"/>
-      <c r="G90" s="8"/>
-      <c r="H90" s="9"/>
-      <c r="I90" s="10"/>
-      <c r="J90" s="7"/>
-    </row>
-    <row r="91" ht="12.8">
-      <c r="A91" s="6"/>
-      <c r="B91" s="7"/>
-      <c r="C91" s="7"/>
-      <c r="D91" s="7"/>
-      <c r="E91" s="7"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="9"/>
-      <c r="I91" s="10"/>
-      <c r="J91" s="7"/>
-    </row>
-    <row r="92" ht="12.8">
-      <c r="A92" s="6"/>
-      <c r="B92" s="7"/>
-      <c r="C92" s="7"/>
-      <c r="D92" s="7"/>
-      <c r="E92" s="7"/>
-      <c r="G92" s="8"/>
-      <c r="H92" s="9"/>
-      <c r="I92" s="10"/>
-      <c r="J92" s="7"/>
-    </row>
-    <row r="93" ht="12.8">
-      <c r="A93" s="6"/>
-      <c r="B93" s="7"/>
-      <c r="C93" s="7"/>
-      <c r="D93" s="7"/>
-      <c r="E93" s="7"/>
-      <c r="G93" s="8"/>
-      <c r="H93" s="9"/>
-      <c r="I93" s="10"/>
-      <c r="J93" s="7"/>
-    </row>
-    <row r="94" ht="12.8">
-      <c r="A94" s="6"/>
-      <c r="B94" s="7"/>
-      <c r="C94" s="7"/>
-      <c r="D94" s="7"/>
-      <c r="E94" s="7"/>
-      <c r="G94" s="8"/>
-      <c r="H94" s="9"/>
-      <c r="I94" s="10"/>
-      <c r="J94" s="7"/>
-    </row>
-    <row r="95" ht="12.8">
-      <c r="A95" s="6"/>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="7"/>
-      <c r="E95" s="7"/>
-      <c r="G95" s="8"/>
-      <c r="H95" s="9"/>
-      <c r="I95" s="10"/>
-      <c r="J95" s="7"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G95" type="list">
-      <formula1>部署!$A$2:$A999</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G80" type="list">
+      <formula1>部署!$A$2:$A991</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H95" type="list">
-      <formula1>役職!$A$2:$A999</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H80" type="list">
+      <formula1>役職!$A$2:$A991</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1876,8 +1747,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" ht="13.8">
-      <c r="A3" s="12" t="s">
+    <row r="3" ht="15.75" customHeight="true">
+      <c r="A3" s="13" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1888,30 +1759,6 @@
     </row>
     <row r="5" ht="15.75" customHeight="true">
       <c r="A5" s="13"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="true">
-      <c r="A6" s="13"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="true">
-      <c r="A7" s="13"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="true">
-      <c r="A8" s="13"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="true">
-      <c r="A9" s="13"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="true">
-      <c r="A10" s="13"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="true">
-      <c r="A11" s="13"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="true">
-      <c r="A12" s="13"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="true">
-      <c r="A13" s="13"/>
     </row>
   </sheetData>
   <printOptions gridLinesSet="true"/>
@@ -1942,36 +1789,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" ht="12.8">
+    <row r="3" ht="15.75" customHeight="true">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="true">
-      <c r="A4" s="1" t="s">
+    <row r="4">
+      <c r="A4" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="true">
-      <c r="A5" s="1"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="true">
-      <c r="A6" s="1"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="true">
-      <c r="A7" s="1"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="true">
-      <c r="A8" s="1"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="true">
-      <c r="A9" s="1"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="true">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="true">
-      <c r="A11" s="1"/>
     </row>
   </sheetData>
   <printOptions gridLinesSet="true"/>

</xml_diff>

<commit_message>
getlist not null positions fixed
</commit_message>
<xml_diff>
--- a/employee_list.xlsx
+++ b/employee_list.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t xml:space="preserve">社員番号</t>
   </si>
@@ -199,6 +199,30 @@
   </si>
   <si>
     <t>admin@gmail.com</t>
+  </si>
+  <si>
+    <t>DK0003</t>
+  </si>
+  <si>
+    <t>Cat123</t>
+  </si>
+  <si>
+    <t>rinatmambedsatlepeso@gmail.com</t>
+  </si>
+  <si>
+    <t>DK00111</t>
+  </si>
+  <si>
+    <t>Mambetlepesov</t>
+  </si>
+  <si>
+    <t>9998991123211</t>
+  </si>
+  <si>
+    <t>suhrob8@gmail.com</t>
+  </si>
+  <si>
+    <t>admin23@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -715,45 +739,45 @@
     </row>
     <row r="2" ht="12.8">
       <c r="A2" s="6" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" ht="12.8">
       <c r="A3" s="6" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>15</v>
@@ -765,30 +789,30 @@
         <v>15</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" ht="12.8">
       <c r="A4" s="6" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>14</v>
@@ -797,16 +821,16 @@
         <v>15</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" ht="12.8">
@@ -820,7 +844,7 @@
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>14</v>
@@ -829,48 +853,48 @@
         <v>15</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>51</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" ht="12.8">
       <c r="A6" s="6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" ht="12.8">
@@ -887,22 +911,22 @@
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>30</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="12.8">
@@ -1532,190 +1556,14 @@
       <c r="I64" s="10"/>
       <c r="J64" s="7"/>
     </row>
-    <row r="65" ht="12.8">
-      <c r="A65" s="6"/>
-      <c r="B65" s="7"/>
-      <c r="C65" s="7"/>
-      <c r="D65" s="7"/>
-      <c r="E65" s="7"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="9"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="7"/>
-    </row>
-    <row r="66" ht="12.8">
-      <c r="A66" s="6"/>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="9"/>
-      <c r="I66" s="10"/>
-      <c r="J66" s="7"/>
-    </row>
-    <row r="67" ht="12.8">
-      <c r="A67" s="6"/>
-      <c r="B67" s="7"/>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7"/>
-      <c r="E67" s="7"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="9"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="7"/>
-    </row>
-    <row r="68" ht="12.8">
-      <c r="A68" s="6"/>
-      <c r="B68" s="7"/>
-      <c r="C68" s="7"/>
-      <c r="D68" s="7"/>
-      <c r="E68" s="7"/>
-      <c r="G68" s="8"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="10"/>
-      <c r="J68" s="7"/>
-    </row>
-    <row r="69" ht="12.8">
-      <c r="A69" s="6"/>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="7"/>
-      <c r="E69" s="7"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="7"/>
-    </row>
-    <row r="70" ht="12.8">
-      <c r="A70" s="6"/>
-      <c r="B70" s="7"/>
-      <c r="C70" s="7"/>
-      <c r="D70" s="7"/>
-      <c r="E70" s="7"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="9"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="7"/>
-    </row>
-    <row r="71" ht="12.8">
-      <c r="A71" s="6"/>
-      <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-      <c r="D71" s="7"/>
-      <c r="E71" s="7"/>
-      <c r="G71" s="8"/>
-      <c r="H71" s="9"/>
-      <c r="I71" s="10"/>
-      <c r="J71" s="7"/>
-    </row>
-    <row r="72" ht="12.8">
-      <c r="A72" s="6"/>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
-      <c r="E72" s="7"/>
-      <c r="G72" s="8"/>
-      <c r="H72" s="9"/>
-      <c r="I72" s="10"/>
-      <c r="J72" s="7"/>
-    </row>
-    <row r="73" ht="12.8">
-      <c r="A73" s="6"/>
-      <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-      <c r="D73" s="7"/>
-      <c r="E73" s="7"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="9"/>
-      <c r="I73" s="10"/>
-      <c r="J73" s="7"/>
-    </row>
-    <row r="74" ht="12.8">
-      <c r="A74" s="6"/>
-      <c r="B74" s="7"/>
-      <c r="C74" s="7"/>
-      <c r="D74" s="7"/>
-      <c r="E74" s="7"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="9"/>
-      <c r="I74" s="10"/>
-      <c r="J74" s="7"/>
-    </row>
-    <row r="75" ht="12.8">
-      <c r="A75" s="6"/>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
-      <c r="E75" s="7"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="9"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="7"/>
-    </row>
-    <row r="76" ht="12.8">
-      <c r="A76" s="6"/>
-      <c r="B76" s="7"/>
-      <c r="C76" s="7"/>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
-      <c r="G76" s="8"/>
-      <c r="H76" s="9"/>
-      <c r="I76" s="10"/>
-      <c r="J76" s="7"/>
-    </row>
-    <row r="77" ht="12.8">
-      <c r="A77" s="6"/>
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="7"/>
-      <c r="E77" s="7"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="9"/>
-      <c r="I77" s="10"/>
-      <c r="J77" s="7"/>
-    </row>
-    <row r="78" ht="12.8">
-      <c r="A78" s="6"/>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="7"/>
-      <c r="E78" s="7"/>
-      <c r="G78" s="8"/>
-      <c r="H78" s="9"/>
-      <c r="I78" s="10"/>
-      <c r="J78" s="7"/>
-    </row>
-    <row r="79" ht="12.8">
-      <c r="A79" s="6"/>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="7"/>
-      <c r="E79" s="7"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="9"/>
-      <c r="I79" s="10"/>
-      <c r="J79" s="7"/>
-    </row>
-    <row r="80" ht="12.8">
-      <c r="A80" s="6"/>
-      <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="7"/>
-      <c r="E80" s="7"/>
-      <c r="G80" s="8"/>
-      <c r="H80" s="9"/>
-      <c r="I80" s="10"/>
-      <c r="J80" s="7"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G80" type="list">
-      <formula1>部署!$A$2:$A991</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="G2:G64" type="list">
+      <formula1>部署!$A$2:$A989</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H80" type="list">
-      <formula1>役職!$A$2:$A991</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showErrorMessage="true" sqref="H2:H64" type="list">
+      <formula1>役職!$A$2:$A989</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1744,21 +1592,11 @@
     </row>
     <row r="2" ht="13.8">
       <c r="A2" s="12" t="s">
-        <v>41</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="true">
-      <c r="A3" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="true">
-      <c r="A4" s="13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="true">
-      <c r="A5" s="13"/>
+      <c r="A3" s="13"/>
     </row>
   </sheetData>
   <printOptions gridLinesSet="true"/>
@@ -1786,17 +1624,7 @@
     </row>
     <row r="2" ht="13.8">
       <c r="A2" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="true">
-      <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>